<commit_message>
Add public release version
</commit_message>
<xml_diff>
--- a/data/human_baseline_annotations/annotation_annotator1.xlsx
+++ b/data/human_baseline_annotations/annotation_annotator1.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/railey/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/railey/Documents/pacute/pacute-bench/data/human_baseline_annotations/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DF18048-F555-1041-B66D-FDCAA0F964A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="1800" windowWidth="10440" windowHeight="16660" firstSheet="9" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="1800" windowWidth="34020" windowHeight="20060" firstSheet="6" activeTab="17" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>

</xml_diff>